<commit_message>
[NCBI Daily] 2026-07-14 pipeline results
</commit_message>
<xml_diff>
--- a/results/2026-07-14/NCBI_Eukaryota_Taxonomy_Summary.xlsx
+++ b/results/2026-07-14/NCBI_Eukaryota_Taxonomy_Summary.xlsx
@@ -466,10 +466,10 @@
         <v>1190</v>
       </c>
       <c r="E2" t="n">
-        <v>41921</v>
+        <v>41924</v>
       </c>
       <c r="F2" t="n">
-        <v>765222</v>
+        <v>765262</v>
       </c>
     </row>
     <row r="3">
@@ -493,7 +493,7 @@
         <v>14606</v>
       </c>
       <c r="F3" t="n">
-        <v>215342</v>
+        <v>215346</v>
       </c>
     </row>
     <row r="4">
@@ -517,7 +517,7 @@
         <v>5306</v>
       </c>
       <c r="F4" t="n">
-        <v>77179</v>
+        <v>77180</v>
       </c>
     </row>
     <row r="5">
@@ -541,7 +541,7 @@
         <v>1632</v>
       </c>
       <c r="F5" t="n">
-        <v>56142</v>
+        <v>56159</v>
       </c>
     </row>
     <row r="6">
@@ -565,7 +565,7 @@
         <v>4791</v>
       </c>
       <c r="F6" t="n">
-        <v>52687</v>
+        <v>52690</v>
       </c>
     </row>
     <row r="7">
@@ -589,7 +589,7 @@
         <v>1744</v>
       </c>
       <c r="F7" t="n">
-        <v>41560</v>
+        <v>41563</v>
       </c>
     </row>
     <row r="8">
@@ -634,10 +634,10 @@
         <v>482</v>
       </c>
       <c r="E9" t="n">
-        <v>4081</v>
+        <v>4080</v>
       </c>
       <c r="F9" t="n">
-        <v>32026</v>
+        <v>32028</v>
       </c>
     </row>
     <row r="10">
@@ -661,7 +661,7 @@
         <v>1643</v>
       </c>
       <c r="F10" t="n">
-        <v>25013</v>
+        <v>25015</v>
       </c>
     </row>
     <row r="11">
@@ -709,7 +709,7 @@
         <v>623</v>
       </c>
       <c r="F12" t="n">
-        <v>14615</v>
+        <v>14620</v>
       </c>
     </row>
     <row r="13">
@@ -781,7 +781,7 @@
         <v>904</v>
       </c>
       <c r="F15" t="n">
-        <v>11819</v>
+        <v>11820</v>
       </c>
     </row>
     <row r="16">
@@ -829,7 +829,7 @@
         <v>1167</v>
       </c>
       <c r="F17" t="n">
-        <v>11710</v>
+        <v>11711</v>
       </c>
     </row>
     <row r="18">
@@ -925,7 +925,7 @@
         <v>876</v>
       </c>
       <c r="F21" t="n">
-        <v>9724</v>
+        <v>9726</v>
       </c>
     </row>
     <row r="22">
@@ -997,7 +997,7 @@
         <v>637</v>
       </c>
       <c r="F24" t="n">
-        <v>8343</v>
+        <v>8346</v>
       </c>
     </row>
     <row r="25">
@@ -1045,7 +1045,7 @@
         <v>979</v>
       </c>
       <c r="F26" t="n">
-        <v>6989</v>
+        <v>6994</v>
       </c>
     </row>
     <row r="27">
@@ -1165,7 +1165,7 @@
         <v>909</v>
       </c>
       <c r="F31" t="n">
-        <v>4807</v>
+        <v>4830</v>
       </c>
     </row>
     <row r="32">
@@ -1213,7 +1213,7 @@
         <v>316</v>
       </c>
       <c r="F33" t="n">
-        <v>4485</v>
+        <v>4486</v>
       </c>
     </row>
     <row r="34">
@@ -1405,7 +1405,7 @@
         <v>524</v>
       </c>
       <c r="F41" t="n">
-        <v>2843</v>
+        <v>2844</v>
       </c>
     </row>
     <row r="42">
@@ -1963,46 +1963,46 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Discosea</t>
+          <t>Ciliophora</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>unclassified Discosea class</t>
+          <t>Spirotrichea</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D65" t="n">
-        <v>10</v>
+        <v>62</v>
       </c>
       <c r="E65" t="n">
-        <v>31</v>
+        <v>285</v>
       </c>
       <c r="F65" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Ciliophora</t>
+          <t>Discosea</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Spirotrichea</t>
+          <t>unclassified Discosea class</t>
         </is>
       </c>
       <c r="C66" t="n">
+        <v>5</v>
+      </c>
+      <c r="D66" t="n">
         <v>10</v>
       </c>
-      <c r="D66" t="n">
-        <v>62</v>
-      </c>
       <c r="E66" t="n">
-        <v>285</v>
+        <v>31</v>
       </c>
       <c r="F66" t="n">
         <v>1332</v>
@@ -2269,7 +2269,7 @@
         <v>87</v>
       </c>
       <c r="F77" t="n">
-        <v>1045</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="78">
@@ -2797,7 +2797,7 @@
         <v>36</v>
       </c>
       <c r="F99" t="n">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="100">
@@ -3565,7 +3565,7 @@
         <v>31</v>
       </c>
       <c r="F131" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="132">
@@ -3733,7 +3733,7 @@
         <v>13</v>
       </c>
       <c r="F138" t="n">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="139">

</xml_diff>